<commit_message>
now excel erros upload show honge teacher ko kaha error aa raha hai konse row pe column pe
</commit_message>
<xml_diff>
--- a/backend/exports/attendance/ComputerEngineering_2025-2026_A_DataStructure_Attendance.xlsx
+++ b/backend/exports/attendance/ComputerEngineering_2025-2026_A_DataStructure_Attendance.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="24">
   <si>
     <t>Watumull Institute of Electronics Engineering &amp; Computer Technology</t>
   </si>
@@ -37,6 +37,9 @@
     <t>2026-07-08</t>
   </si>
   <si>
+    <t>2026-07-09</t>
+  </si>
+  <si>
     <t>Total Present</t>
   </si>
   <si>
@@ -61,6 +64,9 @@
     <t>Diya Mehta</t>
   </si>
   <si>
+    <t>50.00%</t>
+  </si>
+  <si>
     <t>Esha Singh</t>
   </si>
   <si>
@@ -68,9 +74,6 @@
   </si>
   <si>
     <t>Gita Verma</t>
-  </si>
-  <si>
-    <t>0.00%</t>
   </si>
   <si>
     <t>Harsh Reddy</t>
@@ -511,14 +514,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="3" max="4" width="12" customWidth="1"/>
+    <col min="5" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -566,7 +569,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="20" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>5</v>
       </c>
@@ -585,13 +588,16 @@
       <c r="F6" s="5" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6">
         <v>1</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C7" s="7">
         <v>1</v>
@@ -600,38 +606,44 @@
         <v>1</v>
       </c>
       <c r="E7" s="5">
-        <v>0</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F7" s="5">
+        <v>0</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="6">
         <v>2</v>
       </c>
       <c r="B8" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="7">
+        <v>1</v>
+      </c>
+      <c r="D8" s="5">
+        <v>1</v>
+      </c>
+      <c r="E8" s="5">
+        <v>2</v>
+      </c>
+      <c r="F8" s="5">
+        <v>0</v>
+      </c>
+      <c r="G8" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="7">
-        <v>1</v>
-      </c>
-      <c r="D8" s="5">
-        <v>1</v>
-      </c>
-      <c r="E8" s="5">
-        <v>0</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6">
         <v>3</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C9" s="7">
         <v>1</v>
@@ -640,38 +652,44 @@
         <v>1</v>
       </c>
       <c r="E9" s="5">
-        <v>0</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F9" s="5">
+        <v>0</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="6">
         <v>4</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C10" s="7">
         <v>1</v>
       </c>
       <c r="D10" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" s="5">
-        <v>0</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="F10" s="5">
+        <v>1</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="6">
         <v>5</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C11" s="7">
         <v>1</v>
@@ -680,18 +698,21 @@
         <v>1</v>
       </c>
       <c r="E11" s="5">
-        <v>0</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F11" s="5">
+        <v>0</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6">
         <v>6</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C12" s="7">
         <v>1</v>
@@ -700,58 +721,67 @@
         <v>1</v>
       </c>
       <c r="E12" s="5">
-        <v>0</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F12" s="5">
+        <v>0</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="6">
         <v>7</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C13" s="7">
         <v>0</v>
       </c>
       <c r="D13" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" s="5">
         <v>1</v>
       </c>
-      <c r="F13" s="9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F13" s="5">
+        <v>1</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6">
         <v>8</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C14" s="7">
         <v>0</v>
       </c>
       <c r="D14" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" s="5">
         <v>1</v>
       </c>
-      <c r="F14" s="9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F14" s="5">
+        <v>1</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="6">
         <v>9</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C15" s="7">
         <v>1</v>
@@ -760,18 +790,21 @@
         <v>1</v>
       </c>
       <c r="E15" s="5">
-        <v>0</v>
-      </c>
-      <c r="F15" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F15" s="5">
+        <v>0</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6">
         <v>10</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C16" s="7">
         <v>1</v>
@@ -780,10 +813,13 @@
         <v>1</v>
       </c>
       <c r="E16" s="5">
-        <v>0</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>12</v>
+        <v>2</v>
+      </c>
+      <c r="F16" s="5">
+        <v>0</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>